<commit_message>
auto: update dengue data 2026-05-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -465,7 +465,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -557,7 +557,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -577,10 +577,10 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -646,10 +646,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D10" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12" t="n">
         <v>62</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D14" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -787,7 +787,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -833,7 +833,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -853,7 +853,7 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" t="n">
         <v>33</v>
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -922,7 +922,7 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D22" t="n">
         <v>52</v>
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -968,7 +968,7 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D24" t="n">
         <v>56</v>
@@ -991,10 +991,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1017,7 +1017,7 @@
         <v>18</v>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E26" t="n">
         <v>14129</v>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1060,10 +1060,10 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D29" t="n">
         <v>23</v>
@@ -1109,7 +1109,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1129,10 +1129,10 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D31" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" t="n">
         <v>37</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D34" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1267,10 +1267,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1292,10 +1292,10 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E38" t="n">
         <v>17390</v>
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1417,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D44" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1470,7 +1470,7 @@
         <v>62</v>
       </c>
       <c r="D45" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D46" t="n">
         <v>55</v>
@@ -1517,7 +1517,7 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D47" t="n">
         <v>47</v>
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D48" t="n">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1620,7 +1620,7 @@
         <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1670,7 +1670,7 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1717,10 +1717,10 @@
         <v>6459</v>
       </c>
       <c r="C55" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D55" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1742,7 +1742,7 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D56" t="n">
         <v>38</v>
@@ -1770,7 +1770,7 @@
         <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1792,7 +1792,7 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D58" t="n">
         <v>35</v>
@@ -1845,7 +1845,7 @@
         <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1867,10 +1867,10 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D61" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1963,12 +1963,14 @@
           <t>2026-04</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
+      <c r="B65" t="n">
+        <v>2918</v>
+      </c>
       <c r="C65" t="n">
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>

</xml_diff>

<commit_message>
auto: update dengue data 2026-06-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,10 +508,10 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" t="n">
         <v>10289</v>
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -557,7 +557,7 @@
         <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -580,7 +580,7 @@
         <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -603,7 +603,7 @@
         <v>20</v>
       </c>
       <c r="D8" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -646,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D10" t="n">
         <v>81</v>
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -692,10 +692,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -715,10 +715,10 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D13" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -787,7 +787,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D21" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -922,10 +922,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
+        <v>54</v>
+      </c>
+      <c r="D22" t="n">
         <v>53</v>
-      </c>
-      <c r="D22" t="n">
-        <v>52</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -948,7 +948,7 @@
         <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -968,7 +968,7 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D24" t="n">
         <v>56</v>
@@ -991,10 +991,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
         <v>26</v>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27" t="n">
         <v>33</v>
@@ -1063,7 +1063,7 @@
         <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" t="n">
         <v>23</v>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
+        <v>37</v>
+      </c>
+      <c r="D32" t="n">
         <v>38</v>
-      </c>
-      <c r="D32" t="n">
-        <v>37</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D33" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D34" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1267,10 +1267,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1417,10 +1417,10 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E43" t="n">
         <v>16505</v>
@@ -1442,7 +1442,7 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D44" t="n">
         <v>63</v>
@@ -1470,7 +1470,7 @@
         <v>62</v>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D46" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D47" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D48" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1595,7 +1595,7 @@
         <v>12</v>
       </c>
       <c r="D50" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1670,7 +1670,7 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1717,10 +1717,10 @@
         <v>6459</v>
       </c>
       <c r="C55" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1745,7 +1745,7 @@
         <v>17</v>
       </c>
       <c r="D56" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1792,7 +1792,7 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D58" t="n">
         <v>35</v>
@@ -1845,7 +1845,7 @@
         <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1870,7 +1870,7 @@
         <v>9</v>
       </c>
       <c r="D61" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1942,10 +1942,10 @@
         <v>3085</v>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D64" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1989,14 +1989,35 @@
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
+      <c r="C66" t="n">
+        <v>6</v>
+      </c>
+      <c r="D66" t="n">
+        <v>28</v>
+      </c>
       <c r="E66" t="n">
-        <v>56</v>
+        <v>3462</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>85</v>
+        <v>3870</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>82</v>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="n">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update dengue data 2026-06-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -465,7 +465,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
         <v>25</v>
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -554,10 +554,10 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -577,10 +577,10 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -646,10 +646,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D10" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -695,7 +695,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -853,7 +853,7 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D19" t="n">
         <v>33</v>
@@ -879,7 +879,7 @@
         <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
+        <v>38</v>
+      </c>
+      <c r="D21" t="n">
         <v>37</v>
-      </c>
-      <c r="D21" t="n">
-        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -922,10 +922,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" t="n">
         <v>54</v>
-      </c>
-      <c r="D22" t="n">
-        <v>53</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D23" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -991,10 +991,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D25" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1014,10 +1014,10 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E26" t="n">
         <v>14129</v>
@@ -1037,10 +1037,10 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D27" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -1060,10 +1060,10 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1083,10 +1083,10 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1109,7 +1109,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
+        <v>41</v>
+      </c>
+      <c r="D32" t="n">
         <v>37</v>
-      </c>
-      <c r="D32" t="n">
-        <v>38</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D34" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D36" t="n">
         <v>51</v>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D37" t="n">
         <v>32</v>
@@ -1342,10 +1342,10 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1420,7 +1420,7 @@
         <v>25</v>
       </c>
       <c r="D43" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E43" t="n">
         <v>16505</v>
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D45" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D46" t="n">
         <v>56</v>
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D47" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D48" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1592,10 +1592,10 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D50" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
@@ -1667,10 +1667,10 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1742,10 +1742,10 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1770,7 +1770,7 @@
         <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1792,7 +1792,7 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D58" t="n">
         <v>35</v>
@@ -1820,7 +1820,7 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
@@ -1870,7 +1870,7 @@
         <v>9</v>
       </c>
       <c r="D61" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1942,10 +1942,10 @@
         <v>3085</v>
       </c>
       <c r="C64" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1993,7 +1993,7 @@
         <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>

</xml_diff>

<commit_message>
auto: update dengue data 2026-07-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -474,7 +474,7 @@
         <v>3129.2189</v>
       </c>
       <c r="G2" t="n">
-        <v>4016</v>
+        <v>4403</v>
       </c>
     </row>
     <row r="3">
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -497,7 +497,7 @@
         <v>2981.6049</v>
       </c>
       <c r="G3" t="n">
-        <v>5137</v>
+        <v>5913</v>
       </c>
     </row>
     <row r="4">
@@ -520,7 +520,7 @@
         <v>3208.6276</v>
       </c>
       <c r="G4" t="n">
-        <v>6699</v>
+        <v>7598</v>
       </c>
     </row>
     <row r="5">
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -543,7 +543,7 @@
         <v>2849.3583</v>
       </c>
       <c r="G5" t="n">
-        <v>4463</v>
+        <v>4811</v>
       </c>
     </row>
     <row r="6">
@@ -554,10 +554,10 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -566,7 +566,7 @@
         <v>2184.4783</v>
       </c>
       <c r="G6" t="n">
-        <v>4546</v>
+        <v>4792</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>2911.5361</v>
       </c>
       <c r="G7" t="n">
-        <v>4369</v>
+        <v>4905</v>
       </c>
     </row>
     <row r="8">
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -612,7 +612,7 @@
         <v>4433.2881</v>
       </c>
       <c r="G8" t="n">
-        <v>5056</v>
+        <v>5539</v>
       </c>
     </row>
     <row r="9">
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -635,7 +635,7 @@
         <v>9340.807000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>5463</v>
+        <v>5929</v>
       </c>
     </row>
     <row r="10">
@@ -646,10 +646,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D10" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -658,7 +658,7 @@
         <v>18977.9464</v>
       </c>
       <c r="G10" t="n">
-        <v>5855</v>
+        <v>6357</v>
       </c>
     </row>
     <row r="11">
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -681,7 +681,7 @@
         <v>25545.1687</v>
       </c>
       <c r="G11" t="n">
-        <v>6830</v>
+        <v>7235</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12" t="n">
         <v>64</v>
@@ -704,7 +704,7 @@
         <v>11923.5522</v>
       </c>
       <c r="G12" t="n">
-        <v>6229</v>
+        <v>6668</v>
       </c>
     </row>
     <row r="13">
@@ -727,7 +727,7 @@
         <v>4663.8559</v>
       </c>
       <c r="G13" t="n">
-        <v>5617</v>
+        <v>6239</v>
       </c>
     </row>
     <row r="14">
@@ -741,7 +741,7 @@
         <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -750,7 +750,7 @@
         <v>2851.1882</v>
       </c>
       <c r="G14" t="n">
-        <v>5713</v>
+        <v>6117</v>
       </c>
     </row>
     <row r="15">
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -773,7 +773,7 @@
         <v>2366.7911</v>
       </c>
       <c r="G15" t="n">
-        <v>4335</v>
+        <v>4745</v>
       </c>
     </row>
     <row r="16">
@@ -796,7 +796,7 @@
         <v>2598.8767</v>
       </c>
       <c r="G16" t="n">
-        <v>7246</v>
+        <v>7667</v>
       </c>
     </row>
     <row r="17">
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -819,7 +819,7 @@
         <v>2548.3312</v>
       </c>
       <c r="G17" t="n">
-        <v>5613</v>
+        <v>6154</v>
       </c>
     </row>
     <row r="18">
@@ -833,7 +833,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -842,7 +842,7 @@
         <v>1997.5654</v>
       </c>
       <c r="G18" t="n">
-        <v>4745</v>
+        <v>5267</v>
       </c>
     </row>
     <row r="19">
@@ -856,7 +856,7 @@
         <v>18</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -865,7 +865,7 @@
         <v>3072.4912</v>
       </c>
       <c r="G19" t="n">
-        <v>4053</v>
+        <v>4768</v>
       </c>
     </row>
     <row r="20">
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -888,7 +888,7 @@
         <v>4101.412</v>
       </c>
       <c r="G20" t="n">
-        <v>6549</v>
+        <v>7618</v>
       </c>
     </row>
     <row r="21">
@@ -902,7 +902,7 @@
         <v>38</v>
       </c>
       <c r="D21" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -911,7 +911,7 @@
         <v>6089.7509</v>
       </c>
       <c r="G21" t="n">
-        <v>7663</v>
+        <v>8494</v>
       </c>
     </row>
     <row r="22">
@@ -925,7 +925,7 @@
         <v>55</v>
       </c>
       <c r="D22" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -934,7 +934,7 @@
         <v>12615.5129</v>
       </c>
       <c r="G22" t="n">
-        <v>8289</v>
+        <v>8979</v>
       </c>
     </row>
     <row r="23">
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -957,7 +957,7 @@
         <v>19115.2163</v>
       </c>
       <c r="G23" t="n">
-        <v>8785</v>
+        <v>9480</v>
       </c>
     </row>
     <row r="24">
@@ -968,7 +968,7 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D24" t="n">
         <v>56</v>
@@ -980,7 +980,7 @@
         <v>17743.3223</v>
       </c>
       <c r="G24" t="n">
-        <v>9289</v>
+        <v>9845</v>
       </c>
     </row>
     <row r="25">
@@ -991,10 +991,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D25" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1003,7 +1003,7 @@
         <v>4299.3351</v>
       </c>
       <c r="G25" t="n">
-        <v>4520</v>
+        <v>4974</v>
       </c>
     </row>
     <row r="26">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
         <v>25</v>
@@ -1026,7 +1026,7 @@
         <v>3051.7552</v>
       </c>
       <c r="G26" t="n">
-        <v>4432</v>
+        <v>4798</v>
       </c>
     </row>
     <row r="27">
@@ -1037,10 +1037,10 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -1049,7 +1049,7 @@
         <v>3130.4701</v>
       </c>
       <c r="G27" t="n">
-        <v>6233</v>
+        <v>6885</v>
       </c>
     </row>
     <row r="28">
@@ -1063,7 +1063,7 @@
         <v>15</v>
       </c>
       <c r="D28" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1072,7 +1072,7 @@
         <v>2798.3631</v>
       </c>
       <c r="G28" t="n">
-        <v>8913</v>
+        <v>9348</v>
       </c>
     </row>
     <row r="29">
@@ -1083,10 +1083,10 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1095,7 +1095,7 @@
         <v>1858.0278</v>
       </c>
       <c r="G29" t="n">
-        <v>5732</v>
+        <v>6039</v>
       </c>
     </row>
     <row r="30">
@@ -1109,7 +1109,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1118,7 +1118,7 @@
         <v>3090.554</v>
       </c>
       <c r="G30" t="n">
-        <v>6207</v>
+        <v>6711</v>
       </c>
     </row>
     <row r="31">
@@ -1132,7 +1132,7 @@
         <v>27</v>
       </c>
       <c r="D31" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1141,7 +1141,7 @@
         <v>3310.0027</v>
       </c>
       <c r="G31" t="n">
-        <v>5063</v>
+        <v>5541</v>
       </c>
     </row>
     <row r="32">
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D32" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1164,7 +1164,7 @@
         <v>8340.5954</v>
       </c>
       <c r="G32" t="n">
-        <v>7516</v>
+        <v>8574</v>
       </c>
     </row>
     <row r="33">
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D33" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1187,7 +1187,7 @@
         <v>11603.5597</v>
       </c>
       <c r="G33" t="n">
-        <v>7698</v>
+        <v>9101</v>
       </c>
     </row>
     <row r="34">
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D34" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1210,7 +1210,7 @@
         <v>19082.9673</v>
       </c>
       <c r="G34" t="n">
-        <v>6717</v>
+        <v>7299</v>
       </c>
     </row>
     <row r="35">
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1233,7 +1233,7 @@
         <v>13542.0717</v>
       </c>
       <c r="G35" t="n">
-        <v>7616</v>
+        <v>8011</v>
       </c>
     </row>
     <row r="36">
@@ -1244,10 +1244,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D36" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1256,7 +1256,7 @@
         <v>8275.5723</v>
       </c>
       <c r="G36" t="n">
-        <v>7099</v>
+        <v>7745</v>
       </c>
     </row>
     <row r="37">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D37" t="n">
         <v>32</v>
@@ -1279,7 +1279,7 @@
         <v>3525.8816</v>
       </c>
       <c r="G37" t="n">
-        <v>7273</v>
+        <v>7888</v>
       </c>
     </row>
     <row r="38">
@@ -1292,7 +1292,7 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D38" t="n">
         <v>30</v>
@@ -1304,7 +1304,7 @@
         <v>2407.4712</v>
       </c>
       <c r="G38" t="n">
-        <v>5346</v>
+        <v>5887</v>
       </c>
     </row>
     <row r="39">
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1329,7 +1329,7 @@
         <v>2340.3037</v>
       </c>
       <c r="G39" t="n">
-        <v>7445</v>
+        <v>8059</v>
       </c>
     </row>
     <row r="40">
@@ -1342,10 +1342,10 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1354,7 +1354,7 @@
         <v>1849.6489</v>
       </c>
       <c r="G40" t="n">
-        <v>6714</v>
+        <v>7211</v>
       </c>
     </row>
     <row r="41">
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1379,7 +1379,7 @@
         <v>1364.129</v>
       </c>
       <c r="G41" t="n">
-        <v>5552</v>
+        <v>5874</v>
       </c>
     </row>
     <row r="42">
@@ -1404,7 +1404,7 @@
         <v>1592.341</v>
       </c>
       <c r="G42" t="n">
-        <v>3082</v>
+        <v>3498</v>
       </c>
     </row>
     <row r="43">
@@ -1417,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1429,7 +1429,7 @@
         <v>1555.0182</v>
       </c>
       <c r="G43" t="n">
-        <v>2181</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="44">
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D44" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1454,7 +1454,7 @@
         <v>2828.7245</v>
       </c>
       <c r="G44" t="n">
-        <v>3467</v>
+        <v>4652</v>
       </c>
     </row>
     <row r="45">
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D45" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1479,7 +1479,7 @@
         <v>2100.1749</v>
       </c>
       <c r="G45" t="n">
-        <v>3928</v>
+        <v>4483</v>
       </c>
     </row>
     <row r="46">
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D46" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1504,7 +1504,7 @@
         <v>2551.7948</v>
       </c>
       <c r="G46" t="n">
-        <v>3018</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="47">
@@ -1520,7 +1520,7 @@
         <v>53</v>
       </c>
       <c r="D47" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1529,7 +1529,7 @@
         <v>2677.8742</v>
       </c>
       <c r="G47" t="n">
-        <v>3071</v>
+        <v>3449</v>
       </c>
     </row>
     <row r="48">
@@ -1545,7 +1545,7 @@
         <v>34</v>
       </c>
       <c r="D48" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1554,7 +1554,7 @@
         <v>2133.5331</v>
       </c>
       <c r="G48" t="n">
-        <v>2628</v>
+        <v>2863</v>
       </c>
     </row>
     <row r="49">
@@ -1579,7 +1579,7 @@
         <v>1169.4372</v>
       </c>
       <c r="G49" t="n">
-        <v>2087</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="50">
@@ -1592,10 +1592,10 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1604,7 +1604,7 @@
         <v>1067.1823</v>
       </c>
       <c r="G50" t="n">
-        <v>1861</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="51">
@@ -1629,7 +1629,7 @@
         <v>742.0104</v>
       </c>
       <c r="G51" t="n">
-        <v>2000</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="52">
@@ -1654,7 +1654,7 @@
         <v>655.7098</v>
       </c>
       <c r="G52" t="n">
-        <v>2355</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="53">
@@ -1667,10 +1667,10 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1679,7 +1679,7 @@
         <v>602.5579</v>
       </c>
       <c r="G53" t="n">
-        <v>1769</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="54">
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1704,7 +1704,7 @@
         <v>792.1904</v>
       </c>
       <c r="G54" t="n">
-        <v>1765</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="55">
@@ -1729,7 +1729,7 @@
         <v>791.9278</v>
       </c>
       <c r="G55" t="n">
-        <v>2450</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="56">
@@ -1742,10 +1742,10 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D56" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1754,7 +1754,7 @@
         <v>852.0587</v>
       </c>
       <c r="G56" t="n">
-        <v>1892</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="57">
@@ -1770,7 +1770,7 @@
         <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1779,7 +1779,7 @@
         <v>1100.9271</v>
       </c>
       <c r="G57" t="n">
-        <v>2709</v>
+        <v>3055</v>
       </c>
     </row>
     <row r="58">
@@ -1795,7 +1795,7 @@
         <v>22</v>
       </c>
       <c r="D58" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1804,7 +1804,7 @@
         <v>908.633</v>
       </c>
       <c r="G58" t="n">
-        <v>2730</v>
+        <v>3025</v>
       </c>
     </row>
     <row r="59">
@@ -1820,7 +1820,7 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
@@ -1829,7 +1829,7 @@
         <v>771.3006</v>
       </c>
       <c r="G59" t="n">
-        <v>2470</v>
+        <v>2743</v>
       </c>
     </row>
     <row r="60">
@@ -1845,7 +1845,7 @@
         <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1854,7 +1854,7 @@
         <v>668.6939</v>
       </c>
       <c r="G60" t="n">
-        <v>2074</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="61">
@@ -1879,7 +1879,7 @@
         <v>488.4914</v>
       </c>
       <c r="G61" t="n">
-        <v>1760</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="62">
@@ -1895,7 +1895,7 @@
         <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E62" t="n">
         <v>2259</v>
@@ -1904,7 +1904,7 @@
         <v>291.1217</v>
       </c>
       <c r="G62" t="n">
-        <v>1590</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="63">
@@ -1917,7 +1917,7 @@
         <v>3019</v>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D63" t="n">
         <v>30</v>
@@ -1929,7 +1929,7 @@
         <v>279.3269</v>
       </c>
       <c r="G63" t="n">
-        <v>1752</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="64">
@@ -1942,10 +1942,10 @@
         <v>3085</v>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D64" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1954,7 +1954,7 @@
         <v>358.422</v>
       </c>
       <c r="G64" t="n">
-        <v>3485</v>
+        <v>3686</v>
       </c>
     </row>
     <row r="65">
@@ -1979,7 +1979,7 @@
         <v>9.833399999999999</v>
       </c>
       <c r="G65" t="n">
-        <v>3708</v>
+        <v>3992</v>
       </c>
     </row>
     <row r="66">
@@ -1988,19 +1988,21 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
+      <c r="B66" t="n">
+        <v>3747</v>
+      </c>
       <c r="C66" t="n">
         <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>3870</v>
+        <v>4259</v>
       </c>
     </row>
     <row r="67">
@@ -2010,14 +2012,35 @@
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
+      <c r="C67" t="n">
+        <v>9</v>
+      </c>
+      <c r="D67" t="n">
+        <v>21</v>
+      </c>
       <c r="E67" t="n">
-        <v>82</v>
+        <v>3449</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>112</v>
+        <v>2089</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>88</v>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update dengue data 2026-07-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>28</v>
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
         <v>25</v>
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -554,10 +554,10 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -580,7 +580,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,7 +623,7 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D9" t="n">
         <v>55</v>
@@ -646,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D10" t="n">
         <v>78</v>
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
@@ -692,10 +692,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -715,10 +715,10 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D14" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -784,10 +784,10 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D16" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -853,10 +853,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D19" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D21" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -922,10 +922,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D22" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -948,7 +948,7 @@
         <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -971,7 +971,7 @@
         <v>57</v>
       </c>
       <c r="D24" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -991,7 +991,7 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
         <v>31</v>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" t="n">
         <v>25</v>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27" t="n">
         <v>32</v>
@@ -1060,10 +1060,10 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1083,10 +1083,10 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1109,7 +1109,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
+        <v>39</v>
+      </c>
+      <c r="D32" t="n">
         <v>37</v>
-      </c>
-      <c r="D32" t="n">
-        <v>36</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D33" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D34" t="n">
         <v>82</v>
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D36" t="n">
         <v>52</v>
@@ -1270,7 +1270,7 @@
         <v>28</v>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="D40" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1417,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D43" t="n">
         <v>36</v>
@@ -1442,7 +1442,7 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D44" t="n">
         <v>63</v>
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D45" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D46" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1545,7 +1545,7 @@
         <v>34</v>
       </c>
       <c r="D48" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1592,10 +1592,10 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D50" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1620,7 +1620,7 @@
         <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
@@ -1667,10 +1667,10 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1720,7 +1720,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1742,10 +1742,10 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1767,7 +1767,7 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D57" t="n">
         <v>38</v>
@@ -1842,10 +1842,10 @@
         <v>22175</v>
       </c>
       <c r="C60" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D60" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1867,10 +1867,10 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1895,7 +1895,7 @@
         <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E62" t="n">
         <v>2259</v>
@@ -1917,10 +1917,10 @@
         <v>3019</v>
       </c>
       <c r="C63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1942,10 +1942,10 @@
         <v>3085</v>
       </c>
       <c r="C64" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1995,7 +1995,7 @@
         <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>
@@ -2016,7 +2016,7 @@
         <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E67" t="n">
         <v>3449</v>

</xml_diff>

<commit_message>
auto: update dengue data 2026-08-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,10 +462,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -474,7 +474,7 @@
         <v>3129.2189</v>
       </c>
       <c r="G2" t="n">
-        <v>4403</v>
+        <v>4016</v>
       </c>
     </row>
     <row r="3">
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -497,7 +497,7 @@
         <v>2981.6049</v>
       </c>
       <c r="G3" t="n">
-        <v>5913</v>
+        <v>5137</v>
       </c>
     </row>
     <row r="4">
@@ -508,10 +508,10 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
         <v>10289</v>
@@ -520,7 +520,7 @@
         <v>3208.6276</v>
       </c>
       <c r="G4" t="n">
-        <v>7598</v>
+        <v>6699</v>
       </c>
     </row>
     <row r="5">
@@ -534,7 +534,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -543,7 +543,7 @@
         <v>2849.3583</v>
       </c>
       <c r="G5" t="n">
-        <v>4811</v>
+        <v>4463</v>
       </c>
     </row>
     <row r="6">
@@ -557,7 +557,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -566,7 +566,7 @@
         <v>2184.4783</v>
       </c>
       <c r="G6" t="n">
-        <v>4792</v>
+        <v>4546</v>
       </c>
     </row>
     <row r="7">
@@ -580,7 +580,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -589,7 +589,7 @@
         <v>2911.5361</v>
       </c>
       <c r="G7" t="n">
-        <v>4905</v>
+        <v>4369</v>
       </c>
     </row>
     <row r="8">
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="n">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -612,7 +612,7 @@
         <v>4433.2881</v>
       </c>
       <c r="G8" t="n">
-        <v>5539</v>
+        <v>5056</v>
       </c>
     </row>
     <row r="9">
@@ -626,7 +626,7 @@
         <v>35</v>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -635,7 +635,7 @@
         <v>9340.807000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>5929</v>
+        <v>5463</v>
       </c>
     </row>
     <row r="10">
@@ -649,7 +649,7 @@
         <v>59</v>
       </c>
       <c r="D10" t="n">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -658,7 +658,7 @@
         <v>18977.9464</v>
       </c>
       <c r="G10" t="n">
-        <v>6357</v>
+        <v>5855</v>
       </c>
     </row>
     <row r="11">
@@ -669,10 +669,10 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D11" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="E11" t="n">
         <v>62856</v>
@@ -681,7 +681,7 @@
         <v>25545.1687</v>
       </c>
       <c r="G11" t="n">
-        <v>7235</v>
+        <v>6830</v>
       </c>
     </row>
     <row r="12">
@@ -695,7 +695,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -704,7 +704,7 @@
         <v>11923.5522</v>
       </c>
       <c r="G12" t="n">
-        <v>6668</v>
+        <v>6229</v>
       </c>
     </row>
     <row r="13">
@@ -718,7 +718,7 @@
         <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -727,7 +727,7 @@
         <v>4663.8559</v>
       </c>
       <c r="G13" t="n">
-        <v>6239</v>
+        <v>5617</v>
       </c>
     </row>
     <row r="14">
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -750,7 +750,7 @@
         <v>2851.1882</v>
       </c>
       <c r="G14" t="n">
-        <v>6117</v>
+        <v>5713</v>
       </c>
     </row>
     <row r="15">
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -773,7 +773,7 @@
         <v>2366.7911</v>
       </c>
       <c r="G15" t="n">
-        <v>4745</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="16">
@@ -784,10 +784,10 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -796,7 +796,7 @@
         <v>2598.8767</v>
       </c>
       <c r="G16" t="n">
-        <v>7667</v>
+        <v>7246</v>
       </c>
     </row>
     <row r="17">
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -819,7 +819,7 @@
         <v>2548.3312</v>
       </c>
       <c r="G17" t="n">
-        <v>6154</v>
+        <v>5613</v>
       </c>
     </row>
     <row r="18">
@@ -833,7 +833,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -842,7 +842,7 @@
         <v>1997.5654</v>
       </c>
       <c r="G18" t="n">
-        <v>5267</v>
+        <v>4745</v>
       </c>
     </row>
     <row r="19">
@@ -856,7 +856,7 @@
         <v>19</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -865,7 +865,7 @@
         <v>3072.4912</v>
       </c>
       <c r="G19" t="n">
-        <v>4768</v>
+        <v>4053</v>
       </c>
     </row>
     <row r="20">
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -888,7 +888,7 @@
         <v>4101.412</v>
       </c>
       <c r="G20" t="n">
-        <v>7618</v>
+        <v>6549</v>
       </c>
     </row>
     <row r="21">
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D21" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -911,7 +911,7 @@
         <v>6089.7509</v>
       </c>
       <c r="G21" t="n">
-        <v>8494</v>
+        <v>7663</v>
       </c>
     </row>
     <row r="22">
@@ -922,10 +922,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -934,7 +934,7 @@
         <v>12615.5129</v>
       </c>
       <c r="G22" t="n">
-        <v>8979</v>
+        <v>8289</v>
       </c>
     </row>
     <row r="23">
@@ -948,7 +948,7 @@
         <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -957,7 +957,7 @@
         <v>19115.2163</v>
       </c>
       <c r="G23" t="n">
-        <v>9480</v>
+        <v>8785</v>
       </c>
     </row>
     <row r="24">
@@ -971,7 +971,7 @@
         <v>57</v>
       </c>
       <c r="D24" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -980,7 +980,7 @@
         <v>17743.3223</v>
       </c>
       <c r="G24" t="n">
-        <v>9845</v>
+        <v>9289</v>
       </c>
     </row>
     <row r="25">
@@ -994,7 +994,7 @@
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1003,7 +1003,7 @@
         <v>4299.3351</v>
       </c>
       <c r="G25" t="n">
-        <v>4974</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="26">
@@ -1014,10 +1014,10 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
         <v>14129</v>
@@ -1026,7 +1026,7 @@
         <v>3051.7552</v>
       </c>
       <c r="G26" t="n">
-        <v>4798</v>
+        <v>4432</v>
       </c>
     </row>
     <row r="27">
@@ -1037,10 +1037,10 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -1049,7 +1049,7 @@
         <v>3130.4701</v>
       </c>
       <c r="G27" t="n">
-        <v>6885</v>
+        <v>6233</v>
       </c>
     </row>
     <row r="28">
@@ -1063,7 +1063,7 @@
         <v>16</v>
       </c>
       <c r="D28" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1072,7 +1072,7 @@
         <v>2798.3631</v>
       </c>
       <c r="G28" t="n">
-        <v>9348</v>
+        <v>8913</v>
       </c>
     </row>
     <row r="29">
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1095,7 +1095,7 @@
         <v>1858.0278</v>
       </c>
       <c r="G29" t="n">
-        <v>6039</v>
+        <v>5732</v>
       </c>
     </row>
     <row r="30">
@@ -1109,7 +1109,7 @@
         <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1118,7 +1118,7 @@
         <v>3090.554</v>
       </c>
       <c r="G30" t="n">
-        <v>6711</v>
+        <v>6207</v>
       </c>
     </row>
     <row r="31">
@@ -1132,7 +1132,7 @@
         <v>27</v>
       </c>
       <c r="D31" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1141,7 +1141,7 @@
         <v>3310.0027</v>
       </c>
       <c r="G31" t="n">
-        <v>5541</v>
+        <v>5063</v>
       </c>
     </row>
     <row r="32">
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D32" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1164,7 +1164,7 @@
         <v>8340.5954</v>
       </c>
       <c r="G32" t="n">
-        <v>8574</v>
+        <v>7516</v>
       </c>
     </row>
     <row r="33">
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D33" t="n">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1187,7 +1187,7 @@
         <v>11603.5597</v>
       </c>
       <c r="G33" t="n">
-        <v>9101</v>
+        <v>7698</v>
       </c>
     </row>
     <row r="34">
@@ -1201,7 +1201,7 @@
         <v>99</v>
       </c>
       <c r="D34" t="n">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1210,7 +1210,7 @@
         <v>19082.9673</v>
       </c>
       <c r="G34" t="n">
-        <v>7299</v>
+        <v>6717</v>
       </c>
     </row>
     <row r="35">
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1233,7 +1233,7 @@
         <v>13542.0717</v>
       </c>
       <c r="G35" t="n">
-        <v>8011</v>
+        <v>7616</v>
       </c>
     </row>
     <row r="36">
@@ -1244,10 +1244,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D36" t="n">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1256,7 +1256,7 @@
         <v>8275.5723</v>
       </c>
       <c r="G36" t="n">
-        <v>7745</v>
+        <v>7099</v>
       </c>
     </row>
     <row r="37">
@@ -1270,7 +1270,7 @@
         <v>28</v>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1279,7 +1279,7 @@
         <v>3525.8816</v>
       </c>
       <c r="G37" t="n">
-        <v>7888</v>
+        <v>7273</v>
       </c>
     </row>
     <row r="38">
@@ -1295,7 +1295,7 @@
         <v>21</v>
       </c>
       <c r="D38" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
         <v>17390</v>
@@ -1304,7 +1304,7 @@
         <v>2407.4712</v>
       </c>
       <c r="G38" t="n">
-        <v>5887</v>
+        <v>5346</v>
       </c>
     </row>
     <row r="39">
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1329,7 +1329,7 @@
         <v>2340.3037</v>
       </c>
       <c r="G39" t="n">
-        <v>8059</v>
+        <v>7445</v>
       </c>
     </row>
     <row r="40">
@@ -1342,10 +1342,10 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1354,7 +1354,7 @@
         <v>1849.6489</v>
       </c>
       <c r="G40" t="n">
-        <v>7211</v>
+        <v>6714</v>
       </c>
     </row>
     <row r="41">
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1379,7 +1379,7 @@
         <v>1364.129</v>
       </c>
       <c r="G41" t="n">
-        <v>5874</v>
+        <v>5552</v>
       </c>
     </row>
     <row r="42">
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1404,7 +1404,7 @@
         <v>1592.341</v>
       </c>
       <c r="G42" t="n">
-        <v>3498</v>
+        <v>3082</v>
       </c>
     </row>
     <row r="43">
@@ -1420,7 +1420,7 @@
         <v>24</v>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
         <v>16505</v>
@@ -1429,7 +1429,7 @@
         <v>1555.0182</v>
       </c>
       <c r="G43" t="n">
-        <v>2875</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="44">
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1454,7 +1454,7 @@
         <v>2828.7245</v>
       </c>
       <c r="G44" t="n">
-        <v>4652</v>
+        <v>3467</v>
       </c>
     </row>
     <row r="45">
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D45" t="n">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1479,7 +1479,7 @@
         <v>2100.1749</v>
       </c>
       <c r="G45" t="n">
-        <v>4483</v>
+        <v>3928</v>
       </c>
     </row>
     <row r="46">
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D46" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1504,7 +1504,7 @@
         <v>2551.7948</v>
       </c>
       <c r="G46" t="n">
-        <v>3434</v>
+        <v>3018</v>
       </c>
     </row>
     <row r="47">
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D47" t="n">
-        <v>48</v>
+        <v>9</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1529,7 +1529,7 @@
         <v>2677.8742</v>
       </c>
       <c r="G47" t="n">
-        <v>3449</v>
+        <v>3071</v>
       </c>
     </row>
     <row r="48">
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D48" t="n">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1554,7 +1554,7 @@
         <v>2133.5331</v>
       </c>
       <c r="G48" t="n">
-        <v>2863</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="49">
@@ -1570,7 +1570,7 @@
         <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E49" t="n">
         <v>10532</v>
@@ -1579,7 +1579,7 @@
         <v>1169.4372</v>
       </c>
       <c r="G49" t="n">
-        <v>2420</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="50">
@@ -1595,7 +1595,7 @@
         <v>13</v>
       </c>
       <c r="D50" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1604,7 +1604,7 @@
         <v>1067.1823</v>
       </c>
       <c r="G50" t="n">
-        <v>2276</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="51">
@@ -1620,7 +1620,7 @@
         <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1629,7 +1629,7 @@
         <v>742.0104</v>
       </c>
       <c r="G51" t="n">
-        <v>2259</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="52">
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E52" t="n">
         <v>5131</v>
@@ -1654,7 +1654,7 @@
         <v>655.7098</v>
       </c>
       <c r="G52" t="n">
-        <v>2625</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="53">
@@ -1667,10 +1667,10 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1679,7 +1679,7 @@
         <v>602.5579</v>
       </c>
       <c r="G53" t="n">
-        <v>2018</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="54">
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1704,7 +1704,7 @@
         <v>792.1904</v>
       </c>
       <c r="G54" t="n">
-        <v>2166</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="55">
@@ -1720,7 +1720,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1729,7 +1729,7 @@
         <v>791.9278</v>
       </c>
       <c r="G55" t="n">
-        <v>2900</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="56">
@@ -1745,7 +1745,7 @@
         <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1754,7 +1754,7 @@
         <v>852.0587</v>
       </c>
       <c r="G56" t="n">
-        <v>2166</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="57">
@@ -1770,7 +1770,7 @@
         <v>25</v>
       </c>
       <c r="D57" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1779,7 +1779,7 @@
         <v>1100.9271</v>
       </c>
       <c r="G57" t="n">
-        <v>3055</v>
+        <v>2709</v>
       </c>
     </row>
     <row r="58">
@@ -1795,7 +1795,7 @@
         <v>22</v>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1804,7 +1804,7 @@
         <v>908.633</v>
       </c>
       <c r="G58" t="n">
-        <v>3025</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="59">
@@ -1820,7 +1820,7 @@
         <v>20</v>
       </c>
       <c r="D59" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
@@ -1829,7 +1829,7 @@
         <v>771.3006</v>
       </c>
       <c r="G59" t="n">
-        <v>2743</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="60">
@@ -1842,10 +1842,10 @@
         <v>22175</v>
       </c>
       <c r="C60" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1854,7 +1854,7 @@
         <v>668.6939</v>
       </c>
       <c r="G60" t="n">
-        <v>2282</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="61">
@@ -1870,7 +1870,7 @@
         <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1879,7 +1879,7 @@
         <v>488.4914</v>
       </c>
       <c r="G61" t="n">
-        <v>2029</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="62">
@@ -1895,7 +1895,7 @@
         <v>8</v>
       </c>
       <c r="D62" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E62" t="n">
         <v>2259</v>
@@ -1904,7 +1904,7 @@
         <v>291.1217</v>
       </c>
       <c r="G62" t="n">
-        <v>1846</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="63">
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1929,7 +1929,7 @@
         <v>279.3269</v>
       </c>
       <c r="G63" t="n">
-        <v>1978</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="64">
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1954,7 +1954,7 @@
         <v>358.422</v>
       </c>
       <c r="G64" t="n">
-        <v>3686</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="65">
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1979,7 +1979,7 @@
         <v>9.833399999999999</v>
       </c>
       <c r="G65" t="n">
-        <v>3992</v>
+        <v>3708</v>
       </c>
     </row>
     <row r="66">
@@ -1995,14 +1995,14 @@
         <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>4259</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="67">
@@ -2011,19 +2011,21 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
+      <c r="B67" t="n">
+        <v>6625</v>
+      </c>
       <c r="C67" t="n">
         <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E67" t="n">
         <v>3449</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>2089</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="68">
@@ -2033,14 +2035,35 @@
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
+      <c r="C68" t="n">
+        <v>14</v>
+      </c>
+      <c r="D68" t="n">
+        <v>100</v>
+      </c>
       <c r="E68" t="n">
-        <v>88</v>
+        <v>4063</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
-        <v>61</v>
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>111</v>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="n">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update dengue data 2026-08-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -465,7 +465,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -474,7 +474,7 @@
         <v>3129.2189</v>
       </c>
       <c r="G2" t="n">
-        <v>4016</v>
+        <v>4403</v>
       </c>
     </row>
     <row r="3">
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -497,7 +497,7 @@
         <v>2981.6049</v>
       </c>
       <c r="G3" t="n">
-        <v>5137</v>
+        <v>5913</v>
       </c>
     </row>
     <row r="4">
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
@@ -520,7 +520,7 @@
         <v>3208.6276</v>
       </c>
       <c r="G4" t="n">
-        <v>6699</v>
+        <v>7598</v>
       </c>
     </row>
     <row r="5">
@@ -543,7 +543,7 @@
         <v>2849.3583</v>
       </c>
       <c r="G5" t="n">
-        <v>4463</v>
+        <v>4811</v>
       </c>
     </row>
     <row r="6">
@@ -566,7 +566,7 @@
         <v>2184.4783</v>
       </c>
       <c r="G6" t="n">
-        <v>4546</v>
+        <v>4792</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>2911.5361</v>
       </c>
       <c r="G7" t="n">
-        <v>4369</v>
+        <v>4905</v>
       </c>
     </row>
     <row r="8">
@@ -600,7 +600,7 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D8" t="n">
         <v>11</v>
@@ -612,7 +612,7 @@
         <v>4433.2881</v>
       </c>
       <c r="G8" t="n">
-        <v>5056</v>
+        <v>5539</v>
       </c>
     </row>
     <row r="9">
@@ -626,7 +626,7 @@
         <v>35</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -635,7 +635,7 @@
         <v>9340.807000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>5463</v>
+        <v>5929</v>
       </c>
     </row>
     <row r="10">
@@ -646,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D10" t="n">
         <v>15</v>
@@ -658,7 +658,7 @@
         <v>18977.9464</v>
       </c>
       <c r="G10" t="n">
-        <v>5855</v>
+        <v>6357</v>
       </c>
     </row>
     <row r="11">
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D11" t="n">
         <v>19</v>
@@ -681,7 +681,7 @@
         <v>25545.1687</v>
       </c>
       <c r="G11" t="n">
-        <v>6830</v>
+        <v>7235</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D12" t="n">
         <v>12</v>
@@ -704,7 +704,7 @@
         <v>11923.5522</v>
       </c>
       <c r="G12" t="n">
-        <v>6229</v>
+        <v>6668</v>
       </c>
     </row>
     <row r="13">
@@ -727,7 +727,7 @@
         <v>4663.8559</v>
       </c>
       <c r="G13" t="n">
-        <v>5617</v>
+        <v>6239</v>
       </c>
     </row>
     <row r="14">
@@ -750,7 +750,7 @@
         <v>2851.1882</v>
       </c>
       <c r="G14" t="n">
-        <v>5713</v>
+        <v>6117</v>
       </c>
     </row>
     <row r="15">
@@ -773,7 +773,7 @@
         <v>2366.7911</v>
       </c>
       <c r="G15" t="n">
-        <v>4335</v>
+        <v>4745</v>
       </c>
     </row>
     <row r="16">
@@ -796,7 +796,7 @@
         <v>2598.8767</v>
       </c>
       <c r="G16" t="n">
-        <v>7246</v>
+        <v>7667</v>
       </c>
     </row>
     <row r="17">
@@ -819,7 +819,7 @@
         <v>2548.3312</v>
       </c>
       <c r="G17" t="n">
-        <v>5613</v>
+        <v>6154</v>
       </c>
     </row>
     <row r="18">
@@ -842,7 +842,7 @@
         <v>1997.5654</v>
       </c>
       <c r="G18" t="n">
-        <v>4745</v>
+        <v>5267</v>
       </c>
     </row>
     <row r="19">
@@ -853,7 +853,7 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D19" t="n">
         <v>6</v>
@@ -865,7 +865,7 @@
         <v>3072.4912</v>
       </c>
       <c r="G19" t="n">
-        <v>4053</v>
+        <v>4768</v>
       </c>
     </row>
     <row r="20">
@@ -879,7 +879,7 @@
         <v>26</v>
       </c>
       <c r="D20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -888,7 +888,7 @@
         <v>4101.412</v>
       </c>
       <c r="G20" t="n">
-        <v>6549</v>
+        <v>7618</v>
       </c>
     </row>
     <row r="21">
@@ -911,7 +911,7 @@
         <v>6089.7509</v>
       </c>
       <c r="G21" t="n">
-        <v>7663</v>
+        <v>8494</v>
       </c>
     </row>
     <row r="22">
@@ -922,7 +922,7 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D22" t="n">
         <v>10</v>
@@ -934,7 +934,7 @@
         <v>12615.5129</v>
       </c>
       <c r="G22" t="n">
-        <v>8289</v>
+        <v>8979</v>
       </c>
     </row>
     <row r="23">
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -957,7 +957,7 @@
         <v>19115.2163</v>
       </c>
       <c r="G23" t="n">
-        <v>8785</v>
+        <v>9480</v>
       </c>
     </row>
     <row r="24">
@@ -968,10 +968,10 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -980,7 +980,7 @@
         <v>17743.3223</v>
       </c>
       <c r="G24" t="n">
-        <v>9289</v>
+        <v>9845</v>
       </c>
     </row>
     <row r="25">
@@ -1003,7 +1003,7 @@
         <v>4299.3351</v>
       </c>
       <c r="G25" t="n">
-        <v>4520</v>
+        <v>4974</v>
       </c>
     </row>
     <row r="26">
@@ -1026,7 +1026,7 @@
         <v>3051.7552</v>
       </c>
       <c r="G26" t="n">
-        <v>4432</v>
+        <v>4798</v>
       </c>
     </row>
     <row r="27">
@@ -1049,7 +1049,7 @@
         <v>3130.4701</v>
       </c>
       <c r="G27" t="n">
-        <v>6233</v>
+        <v>6885</v>
       </c>
     </row>
     <row r="28">
@@ -1072,7 +1072,7 @@
         <v>2798.3631</v>
       </c>
       <c r="G28" t="n">
-        <v>8913</v>
+        <v>9348</v>
       </c>
     </row>
     <row r="29">
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1095,7 +1095,7 @@
         <v>1858.0278</v>
       </c>
       <c r="G29" t="n">
-        <v>5732</v>
+        <v>6039</v>
       </c>
     </row>
     <row r="30">
@@ -1118,7 +1118,7 @@
         <v>3090.554</v>
       </c>
       <c r="G30" t="n">
-        <v>6207</v>
+        <v>6711</v>
       </c>
     </row>
     <row r="31">
@@ -1141,7 +1141,7 @@
         <v>3310.0027</v>
       </c>
       <c r="G31" t="n">
-        <v>5063</v>
+        <v>5541</v>
       </c>
     </row>
     <row r="32">
@@ -1164,7 +1164,7 @@
         <v>8340.5954</v>
       </c>
       <c r="G32" t="n">
-        <v>7516</v>
+        <v>8574</v>
       </c>
     </row>
     <row r="33">
@@ -1178,7 +1178,7 @@
         <v>69</v>
       </c>
       <c r="D33" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1187,7 +1187,7 @@
         <v>11603.5597</v>
       </c>
       <c r="G33" t="n">
-        <v>7698</v>
+        <v>9101</v>
       </c>
     </row>
     <row r="34">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D34" t="n">
         <v>16</v>
@@ -1210,7 +1210,7 @@
         <v>19082.9673</v>
       </c>
       <c r="G34" t="n">
-        <v>6717</v>
+        <v>7299</v>
       </c>
     </row>
     <row r="35">
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1233,7 +1233,7 @@
         <v>13542.0717</v>
       </c>
       <c r="G35" t="n">
-        <v>7616</v>
+        <v>8011</v>
       </c>
     </row>
     <row r="36">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D36" t="n">
         <v>10</v>
@@ -1256,7 +1256,7 @@
         <v>8275.5723</v>
       </c>
       <c r="G36" t="n">
-        <v>7099</v>
+        <v>7745</v>
       </c>
     </row>
     <row r="37">
@@ -1279,7 +1279,7 @@
         <v>3525.8816</v>
       </c>
       <c r="G37" t="n">
-        <v>7273</v>
+        <v>7888</v>
       </c>
     </row>
     <row r="38">
@@ -1292,7 +1292,7 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" t="n">
         <v>6</v>
@@ -1304,7 +1304,7 @@
         <v>2407.4712</v>
       </c>
       <c r="G38" t="n">
-        <v>5346</v>
+        <v>5887</v>
       </c>
     </row>
     <row r="39">
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1329,7 +1329,7 @@
         <v>2340.3037</v>
       </c>
       <c r="G39" t="n">
-        <v>7445</v>
+        <v>8059</v>
       </c>
     </row>
     <row r="40">
@@ -1342,7 +1342,7 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40" t="n">
         <v>5</v>
@@ -1354,7 +1354,7 @@
         <v>1849.6489</v>
       </c>
       <c r="G40" t="n">
-        <v>6714</v>
+        <v>7211</v>
       </c>
     </row>
     <row r="41">
@@ -1379,7 +1379,7 @@
         <v>1364.129</v>
       </c>
       <c r="G41" t="n">
-        <v>5552</v>
+        <v>5874</v>
       </c>
     </row>
     <row r="42">
@@ -1404,7 +1404,7 @@
         <v>1592.341</v>
       </c>
       <c r="G42" t="n">
-        <v>3082</v>
+        <v>3498</v>
       </c>
     </row>
     <row r="43">
@@ -1429,7 +1429,7 @@
         <v>1555.0182</v>
       </c>
       <c r="G43" t="n">
-        <v>2181</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="44">
@@ -1442,7 +1442,7 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D44" t="n">
         <v>12</v>
@@ -1454,7 +1454,7 @@
         <v>2828.7245</v>
       </c>
       <c r="G44" t="n">
-        <v>3467</v>
+        <v>4652</v>
       </c>
     </row>
     <row r="45">
@@ -1467,7 +1467,7 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D45" t="n">
         <v>13</v>
@@ -1479,7 +1479,7 @@
         <v>2100.1749</v>
       </c>
       <c r="G45" t="n">
-        <v>3928</v>
+        <v>4483</v>
       </c>
     </row>
     <row r="46">
@@ -1492,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D46" t="n">
         <v>11</v>
@@ -1504,7 +1504,7 @@
         <v>2551.7948</v>
       </c>
       <c r="G46" t="n">
-        <v>3018</v>
+        <v>3434</v>
       </c>
     </row>
     <row r="47">
@@ -1517,7 +1517,7 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D47" t="n">
         <v>9</v>
@@ -1529,7 +1529,7 @@
         <v>2677.8742</v>
       </c>
       <c r="G47" t="n">
-        <v>3071</v>
+        <v>3449</v>
       </c>
     </row>
     <row r="48">
@@ -1542,7 +1542,7 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D48" t="n">
         <v>9</v>
@@ -1554,7 +1554,7 @@
         <v>2133.5331</v>
       </c>
       <c r="G48" t="n">
-        <v>2628</v>
+        <v>2863</v>
       </c>
     </row>
     <row r="49">
@@ -1579,7 +1579,7 @@
         <v>1169.4372</v>
       </c>
       <c r="G49" t="n">
-        <v>2087</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="50">
@@ -1604,7 +1604,7 @@
         <v>1067.1823</v>
       </c>
       <c r="G50" t="n">
-        <v>1861</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="51">
@@ -1617,10 +1617,10 @@
         <v>3806</v>
       </c>
       <c r="C51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1629,7 +1629,7 @@
         <v>742.0104</v>
       </c>
       <c r="G51" t="n">
-        <v>2000</v>
+        <v>2259</v>
       </c>
     </row>
     <row r="52">
@@ -1654,7 +1654,7 @@
         <v>655.7098</v>
       </c>
       <c r="G52" t="n">
-        <v>2355</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="53">
@@ -1679,7 +1679,7 @@
         <v>602.5579</v>
       </c>
       <c r="G53" t="n">
-        <v>1769</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="54">
@@ -1704,7 +1704,7 @@
         <v>792.1904</v>
       </c>
       <c r="G54" t="n">
-        <v>1765</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="55">
@@ -1729,7 +1729,7 @@
         <v>791.9278</v>
       </c>
       <c r="G55" t="n">
-        <v>2450</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="56">
@@ -1745,7 +1745,7 @@
         <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1754,7 +1754,7 @@
         <v>852.0587</v>
       </c>
       <c r="G56" t="n">
-        <v>1892</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="57">
@@ -1767,10 +1767,10 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1779,7 +1779,7 @@
         <v>1100.9271</v>
       </c>
       <c r="G57" t="n">
-        <v>2709</v>
+        <v>3055</v>
       </c>
     </row>
     <row r="58">
@@ -1792,10 +1792,10 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1804,7 +1804,7 @@
         <v>908.633</v>
       </c>
       <c r="G58" t="n">
-        <v>2730</v>
+        <v>3025</v>
       </c>
     </row>
     <row r="59">
@@ -1829,7 +1829,7 @@
         <v>771.3006</v>
       </c>
       <c r="G59" t="n">
-        <v>2470</v>
+        <v>2743</v>
       </c>
     </row>
     <row r="60">
@@ -1842,7 +1842,7 @@
         <v>22175</v>
       </c>
       <c r="C60" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
@@ -1854,7 +1854,7 @@
         <v>668.6939</v>
       </c>
       <c r="G60" t="n">
-        <v>2074</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="61">
@@ -1867,7 +1867,7 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D61" t="n">
         <v>6</v>
@@ -1879,7 +1879,7 @@
         <v>488.4914</v>
       </c>
       <c r="G61" t="n">
-        <v>1760</v>
+        <v>2029</v>
       </c>
     </row>
     <row r="62">
@@ -1904,7 +1904,7 @@
         <v>291.1217</v>
       </c>
       <c r="G62" t="n">
-        <v>1590</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="63">
@@ -1929,7 +1929,7 @@
         <v>279.3269</v>
       </c>
       <c r="G63" t="n">
-        <v>1752</v>
+        <v>1978</v>
       </c>
     </row>
     <row r="64">
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1954,7 +1954,7 @@
         <v>358.422</v>
       </c>
       <c r="G64" t="n">
-        <v>3485</v>
+        <v>3686</v>
       </c>
     </row>
     <row r="65">
@@ -1979,7 +1979,7 @@
         <v>9.833399999999999</v>
       </c>
       <c r="G65" t="n">
-        <v>3708</v>
+        <v>3992</v>
       </c>
     </row>
     <row r="66">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>3870</v>
+        <v>4259</v>
       </c>
     </row>
     <row r="67">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>1886</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="68">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
-        <v>1372</v>
+        <v>1872</v>
       </c>
     </row>
     <row r="69">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="n">
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update dengue data 2026-09-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -474,7 +474,7 @@
         <v>3129.2189</v>
       </c>
       <c r="G2" t="n">
-        <v>4403</v>
+        <v>4016</v>
       </c>
     </row>
     <row r="3">
@@ -497,7 +497,7 @@
         <v>2981.6049</v>
       </c>
       <c r="G3" t="n">
-        <v>5913</v>
+        <v>5137</v>
       </c>
     </row>
     <row r="4">
@@ -508,7 +508,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
@@ -520,7 +520,7 @@
         <v>3208.6276</v>
       </c>
       <c r="G4" t="n">
-        <v>7598</v>
+        <v>6699</v>
       </c>
     </row>
     <row r="5">
@@ -543,7 +543,7 @@
         <v>2849.3583</v>
       </c>
       <c r="G5" t="n">
-        <v>4811</v>
+        <v>4463</v>
       </c>
     </row>
     <row r="6">
@@ -554,7 +554,7 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
         <v>8</v>
@@ -566,7 +566,7 @@
         <v>2184.4783</v>
       </c>
       <c r="G6" t="n">
-        <v>4792</v>
+        <v>4546</v>
       </c>
     </row>
     <row r="7">
@@ -577,7 +577,7 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="n">
         <v>7</v>
@@ -589,7 +589,7 @@
         <v>2911.5361</v>
       </c>
       <c r="G7" t="n">
-        <v>4905</v>
+        <v>4369</v>
       </c>
     </row>
     <row r="8">
@@ -600,7 +600,7 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
         <v>11</v>
@@ -612,7 +612,7 @@
         <v>4433.2881</v>
       </c>
       <c r="G8" t="n">
-        <v>5539</v>
+        <v>5056</v>
       </c>
     </row>
     <row r="9">
@@ -626,7 +626,7 @@
         <v>35</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -635,7 +635,7 @@
         <v>9340.807000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>5929</v>
+        <v>5463</v>
       </c>
     </row>
     <row r="10">
@@ -646,7 +646,7 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D10" t="n">
         <v>15</v>
@@ -658,7 +658,7 @@
         <v>18977.9464</v>
       </c>
       <c r="G10" t="n">
-        <v>6357</v>
+        <v>5855</v>
       </c>
     </row>
     <row r="11">
@@ -669,7 +669,7 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D11" t="n">
         <v>19</v>
@@ -681,7 +681,7 @@
         <v>25545.1687</v>
       </c>
       <c r="G11" t="n">
-        <v>7235</v>
+        <v>6830</v>
       </c>
     </row>
     <row r="12">
@@ -692,7 +692,7 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" t="n">
         <v>12</v>
@@ -704,7 +704,7 @@
         <v>11923.5522</v>
       </c>
       <c r="G12" t="n">
-        <v>6668</v>
+        <v>6229</v>
       </c>
     </row>
     <row r="13">
@@ -727,7 +727,7 @@
         <v>4663.8559</v>
       </c>
       <c r="G13" t="n">
-        <v>6239</v>
+        <v>5617</v>
       </c>
     </row>
     <row r="14">
@@ -750,7 +750,7 @@
         <v>2851.1882</v>
       </c>
       <c r="G14" t="n">
-        <v>6117</v>
+        <v>5713</v>
       </c>
     </row>
     <row r="15">
@@ -773,7 +773,7 @@
         <v>2366.7911</v>
       </c>
       <c r="G15" t="n">
-        <v>4745</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="16">
@@ -796,7 +796,7 @@
         <v>2598.8767</v>
       </c>
       <c r="G16" t="n">
-        <v>7667</v>
+        <v>7246</v>
       </c>
     </row>
     <row r="17">
@@ -819,7 +819,7 @@
         <v>2548.3312</v>
       </c>
       <c r="G17" t="n">
-        <v>6154</v>
+        <v>5613</v>
       </c>
     </row>
     <row r="18">
@@ -842,7 +842,7 @@
         <v>1997.5654</v>
       </c>
       <c r="G18" t="n">
-        <v>5267</v>
+        <v>4745</v>
       </c>
     </row>
     <row r="19">
@@ -853,7 +853,7 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19" t="n">
         <v>6</v>
@@ -865,7 +865,7 @@
         <v>3072.4912</v>
       </c>
       <c r="G19" t="n">
-        <v>4768</v>
+        <v>4053</v>
       </c>
     </row>
     <row r="20">
@@ -888,7 +888,7 @@
         <v>4101.412</v>
       </c>
       <c r="G20" t="n">
-        <v>7618</v>
+        <v>6549</v>
       </c>
     </row>
     <row r="21">
@@ -911,7 +911,7 @@
         <v>6089.7509</v>
       </c>
       <c r="G21" t="n">
-        <v>8494</v>
+        <v>7663</v>
       </c>
     </row>
     <row r="22">
@@ -922,7 +922,7 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" t="n">
         <v>10</v>
@@ -934,7 +934,7 @@
         <v>12615.5129</v>
       </c>
       <c r="G22" t="n">
-        <v>8979</v>
+        <v>8289</v>
       </c>
     </row>
     <row r="23">
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -957,7 +957,7 @@
         <v>19115.2163</v>
       </c>
       <c r="G23" t="n">
-        <v>9480</v>
+        <v>8785</v>
       </c>
     </row>
     <row r="24">
@@ -968,7 +968,7 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" t="n">
         <v>11</v>
@@ -980,7 +980,7 @@
         <v>17743.3223</v>
       </c>
       <c r="G24" t="n">
-        <v>9845</v>
+        <v>9289</v>
       </c>
     </row>
     <row r="25">
@@ -991,7 +991,7 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" t="n">
         <v>6</v>
@@ -1003,7 +1003,7 @@
         <v>4299.3351</v>
       </c>
       <c r="G25" t="n">
-        <v>4974</v>
+        <v>4520</v>
       </c>
     </row>
     <row r="26">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D26" t="n">
         <v>5</v>
@@ -1026,7 +1026,7 @@
         <v>3051.7552</v>
       </c>
       <c r="G26" t="n">
-        <v>4798</v>
+        <v>4432</v>
       </c>
     </row>
     <row r="27">
@@ -1049,7 +1049,7 @@
         <v>3130.4701</v>
       </c>
       <c r="G27" t="n">
-        <v>6885</v>
+        <v>6233</v>
       </c>
     </row>
     <row r="28">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1072,7 +1072,7 @@
         <v>2798.3631</v>
       </c>
       <c r="G28" t="n">
-        <v>9348</v>
+        <v>8913</v>
       </c>
     </row>
     <row r="29">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" t="n">
         <v>5</v>
@@ -1095,7 +1095,7 @@
         <v>1858.0278</v>
       </c>
       <c r="G29" t="n">
-        <v>6039</v>
+        <v>5732</v>
       </c>
     </row>
     <row r="30">
@@ -1118,7 +1118,7 @@
         <v>3090.554</v>
       </c>
       <c r="G30" t="n">
-        <v>6711</v>
+        <v>6207</v>
       </c>
     </row>
     <row r="31">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D31" t="n">
         <v>6</v>
@@ -1141,7 +1141,7 @@
         <v>3310.0027</v>
       </c>
       <c r="G31" t="n">
-        <v>5541</v>
+        <v>5063</v>
       </c>
     </row>
     <row r="32">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D32" t="n">
         <v>7</v>
@@ -1164,7 +1164,7 @@
         <v>8340.5954</v>
       </c>
       <c r="G32" t="n">
-        <v>8574</v>
+        <v>7516</v>
       </c>
     </row>
     <row r="33">
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D33" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1187,7 +1187,7 @@
         <v>11603.5597</v>
       </c>
       <c r="G33" t="n">
-        <v>9101</v>
+        <v>7698</v>
       </c>
     </row>
     <row r="34">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D34" t="n">
         <v>16</v>
@@ -1210,7 +1210,7 @@
         <v>19082.9673</v>
       </c>
       <c r="G34" t="n">
-        <v>7299</v>
+        <v>6717</v>
       </c>
     </row>
     <row r="35">
@@ -1224,7 +1224,7 @@
         <v>100</v>
       </c>
       <c r="D35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1233,7 +1233,7 @@
         <v>13542.0717</v>
       </c>
       <c r="G35" t="n">
-        <v>8011</v>
+        <v>7616</v>
       </c>
     </row>
     <row r="36">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D36" t="n">
         <v>10</v>
@@ -1256,7 +1256,7 @@
         <v>8275.5723</v>
       </c>
       <c r="G36" t="n">
-        <v>7745</v>
+        <v>7099</v>
       </c>
     </row>
     <row r="37">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D37" t="n">
         <v>6</v>
@@ -1279,7 +1279,7 @@
         <v>3525.8816</v>
       </c>
       <c r="G37" t="n">
-        <v>7888</v>
+        <v>7273</v>
       </c>
     </row>
     <row r="38">
@@ -1304,7 +1304,7 @@
         <v>2407.4712</v>
       </c>
       <c r="G38" t="n">
-        <v>5887</v>
+        <v>5346</v>
       </c>
     </row>
     <row r="39">
@@ -1329,7 +1329,7 @@
         <v>2340.3037</v>
       </c>
       <c r="G39" t="n">
-        <v>8059</v>
+        <v>7445</v>
       </c>
     </row>
     <row r="40">
@@ -1354,7 +1354,7 @@
         <v>1849.6489</v>
       </c>
       <c r="G40" t="n">
-        <v>7211</v>
+        <v>6714</v>
       </c>
     </row>
     <row r="41">
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1379,7 +1379,7 @@
         <v>1364.129</v>
       </c>
       <c r="G41" t="n">
-        <v>5874</v>
+        <v>5552</v>
       </c>
     </row>
     <row r="42">
@@ -1404,7 +1404,7 @@
         <v>1592.341</v>
       </c>
       <c r="G42" t="n">
-        <v>3498</v>
+        <v>3082</v>
       </c>
     </row>
     <row r="43">
@@ -1417,7 +1417,7 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D43" t="n">
         <v>7</v>
@@ -1429,7 +1429,7 @@
         <v>1555.0182</v>
       </c>
       <c r="G43" t="n">
-        <v>2875</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="44">
@@ -1454,7 +1454,7 @@
         <v>2828.7245</v>
       </c>
       <c r="G44" t="n">
-        <v>4652</v>
+        <v>3467</v>
       </c>
     </row>
     <row r="45">
@@ -1470,7 +1470,7 @@
         <v>61</v>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1479,7 +1479,7 @@
         <v>2100.1749</v>
       </c>
       <c r="G45" t="n">
-        <v>4483</v>
+        <v>3928</v>
       </c>
     </row>
     <row r="46">
@@ -1492,7 +1492,7 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D46" t="n">
         <v>11</v>
@@ -1504,7 +1504,7 @@
         <v>2551.7948</v>
       </c>
       <c r="G46" t="n">
-        <v>3434</v>
+        <v>3018</v>
       </c>
     </row>
     <row r="47">
@@ -1517,7 +1517,7 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D47" t="n">
         <v>9</v>
@@ -1529,7 +1529,7 @@
         <v>2677.8742</v>
       </c>
       <c r="G47" t="n">
-        <v>3449</v>
+        <v>3071</v>
       </c>
     </row>
     <row r="48">
@@ -1554,7 +1554,7 @@
         <v>2133.5331</v>
       </c>
       <c r="G48" t="n">
-        <v>2863</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="49">
@@ -1579,7 +1579,7 @@
         <v>1169.4372</v>
       </c>
       <c r="G49" t="n">
-        <v>2420</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="50">
@@ -1592,7 +1592,7 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D50" t="n">
         <v>5</v>
@@ -1604,7 +1604,7 @@
         <v>1067.1823</v>
       </c>
       <c r="G50" t="n">
-        <v>2276</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="51">
@@ -1617,7 +1617,7 @@
         <v>3806</v>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51" t="n">
         <v>4</v>
@@ -1629,7 +1629,7 @@
         <v>742.0104</v>
       </c>
       <c r="G51" t="n">
-        <v>2259</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="52">
@@ -1654,7 +1654,7 @@
         <v>655.7098</v>
       </c>
       <c r="G52" t="n">
-        <v>2625</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="53">
@@ -1679,7 +1679,7 @@
         <v>602.5579</v>
       </c>
       <c r="G53" t="n">
-        <v>2018</v>
+        <v>1769</v>
       </c>
     </row>
     <row r="54">
@@ -1704,7 +1704,7 @@
         <v>792.1904</v>
       </c>
       <c r="G54" t="n">
-        <v>2166</v>
+        <v>1765</v>
       </c>
     </row>
     <row r="55">
@@ -1729,7 +1729,7 @@
         <v>791.9278</v>
       </c>
       <c r="G55" t="n">
-        <v>2900</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="56">
@@ -1742,10 +1742,10 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1754,7 +1754,7 @@
         <v>852.0587</v>
       </c>
       <c r="G56" t="n">
-        <v>2166</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="57">
@@ -1770,7 +1770,7 @@
         <v>24</v>
       </c>
       <c r="D57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1779,7 +1779,7 @@
         <v>1100.9271</v>
       </c>
       <c r="G57" t="n">
-        <v>3055</v>
+        <v>2709</v>
       </c>
     </row>
     <row r="58">
@@ -1792,10 +1792,10 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1804,7 +1804,7 @@
         <v>908.633</v>
       </c>
       <c r="G58" t="n">
-        <v>3025</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="59">
@@ -1829,7 +1829,7 @@
         <v>771.3006</v>
       </c>
       <c r="G59" t="n">
-        <v>2743</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="60">
@@ -1842,7 +1842,7 @@
         <v>22175</v>
       </c>
       <c r="C60" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
@@ -1854,7 +1854,7 @@
         <v>668.6939</v>
       </c>
       <c r="G60" t="n">
-        <v>2282</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="61">
@@ -1879,7 +1879,7 @@
         <v>488.4914</v>
       </c>
       <c r="G61" t="n">
-        <v>2029</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="62">
@@ -1904,7 +1904,7 @@
         <v>291.1217</v>
       </c>
       <c r="G62" t="n">
-        <v>1846</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="63">
@@ -1929,7 +1929,7 @@
         <v>279.3269</v>
       </c>
       <c r="G63" t="n">
-        <v>1978</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="64">
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1954,7 +1954,7 @@
         <v>358.422</v>
       </c>
       <c r="G64" t="n">
-        <v>3686</v>
+        <v>3485</v>
       </c>
     </row>
     <row r="65">
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1979,7 +1979,7 @@
         <v>9.833399999999999</v>
       </c>
       <c r="G65" t="n">
-        <v>3992</v>
+        <v>3708</v>
       </c>
     </row>
     <row r="66">
@@ -1992,7 +1992,7 @@
         <v>3747</v>
       </c>
       <c r="C66" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D66" t="n">
         <v>5</v>
@@ -2002,7 +2002,7 @@
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
-        <v>4259</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="67">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>2089</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="68">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D68" t="n">
         <v>100</v>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
-        <v>1872</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="69">
@@ -2056,14 +2056,35 @@
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
+      <c r="C69" t="n">
+        <v>20</v>
+      </c>
+      <c r="D69" t="n">
+        <v>16</v>
+      </c>
       <c r="E69" t="n">
-        <v>111</v>
+        <v>4067</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="n">
-        <v>87</v>
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>170</v>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="n">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto: update dengue data 2026-09-20
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
         <v>5</v>
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -508,10 +508,10 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>10289</v>
@@ -531,7 +531,7 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" t="n">
         <v>5</v>
@@ -554,10 +554,10 @@
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -577,10 +577,10 @@
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -646,10 +646,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -669,10 +669,10 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E11" t="n">
         <v>62856</v>
@@ -695,7 +695,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -718,7 +718,7 @@
         <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -764,7 +764,7 @@
         <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
         <v>9029</v>
@@ -787,7 +787,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -830,10 +830,10 @@
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -853,10 +853,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -876,10 +876,10 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -922,10 +922,10 @@
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -968,10 +968,10 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -991,10 +991,10 @@
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1014,10 +1014,10 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
         <v>14129</v>
@@ -1040,7 +1040,7 @@
         <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D28" t="n">
         <v>5</v>
@@ -1083,10 +1083,10 @@
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
         <v>10272</v>
@@ -1106,10 +1106,10 @@
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1129,10 +1129,10 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D33" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1198,10 +1198,10 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D34" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1221,10 +1221,10 @@
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D35" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1247,7 +1247,7 @@
         <v>54</v>
       </c>
       <c r="D36" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1267,10 +1267,10 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1292,10 +1292,10 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E38" t="n">
         <v>17390</v>
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1342,10 +1342,10 @@
         <v>5597</v>
       </c>
       <c r="C40" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1417,10 +1417,10 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E43" t="n">
         <v>16505</v>
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D44" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D46" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1570,7 +1570,7 @@
         <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E49" t="n">
         <v>10532</v>
@@ -1592,7 +1592,7 @@
         <v>4700</v>
       </c>
       <c r="C50" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D50" t="n">
         <v>5</v>
@@ -1617,7 +1617,7 @@
         <v>3806</v>
       </c>
       <c r="C51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D51" t="n">
         <v>4</v>
@@ -1667,10 +1667,10 @@
         <v>2700</v>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1720,7 +1720,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1742,10 +1742,10 @@
         <v>10302</v>
       </c>
       <c r="C56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1767,10 +1767,10 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1792,10 +1792,10 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1817,7 +1817,7 @@
         <v>22659</v>
       </c>
       <c r="C59" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D59" t="n">
         <v>5</v>
@@ -1842,10 +1842,10 @@
         <v>22175</v>
       </c>
       <c r="C60" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1867,10 +1867,10 @@
         <v>7539</v>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1992,10 +1992,10 @@
         <v>3747</v>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>
@@ -2034,9 +2034,11 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
+      <c r="B68" t="n">
+        <v>10122</v>
+      </c>
       <c r="C68" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D68" t="n">
         <v>100</v>
@@ -2055,12 +2057,14 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
+      <c r="B69" t="n">
+        <v>13610</v>
+      </c>
       <c r="C69" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D69" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E69" t="n">
         <v>4067</v>

</xml_diff>

<commit_message>
auto: update dengue data 2026-10-05
</commit_message>
<xml_diff>
--- a/dengue_updater/data/processed/master_data.xlsx
+++ b/dengue_updater/data/processed/master_data.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
         <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
         <v>10782</v>
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
         <v>10100</v>
@@ -511,7 +511,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
         <v>10289</v>
@@ -531,10 +531,10 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
         <v>8800</v>
@@ -557,7 +557,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
         <v>9447</v>
@@ -580,7 +580,7 @@
         <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
         <v>13009</v>
@@ -600,10 +600,10 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E8" t="n">
         <v>21349</v>
@@ -623,10 +623,10 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>35620</v>
@@ -646,10 +646,10 @@
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
         <v>55083</v>
@@ -669,10 +669,10 @@
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E11" t="n">
         <v>62856</v>
@@ -695,7 +695,7 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" t="n">
         <v>33621</v>
@@ -718,7 +718,7 @@
         <v>25</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E13" t="n">
         <v>16159</v>
@@ -738,10 +738,10 @@
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E14" t="n">
         <v>11244</v>
@@ -787,7 +787,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
         <v>9603</v>
@@ -810,7 +810,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E17" t="n">
         <v>9781</v>
@@ -830,10 +830,10 @@
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E18" t="n">
         <v>10872</v>
@@ -853,10 +853,10 @@
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
         <v>15980</v>
@@ -879,7 +879,7 @@
         <v>27</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E20" t="n">
         <v>23568</v>
@@ -899,10 +899,10 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>34009</v>
@@ -925,7 +925,7 @@
         <v>56</v>
       </c>
       <c r="D22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E22" t="n">
         <v>57125</v>
@@ -945,10 +945,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
         <v>76590</v>
@@ -968,10 +968,10 @@
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
         <v>74792</v>
@@ -994,7 +994,7 @@
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" t="n">
         <v>20815</v>
@@ -1014,10 +1014,10 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E26" t="n">
         <v>14129</v>
@@ -1040,7 +1040,7 @@
         <v>19</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
         <v>15761</v>
@@ -1060,10 +1060,10 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D28" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" t="n">
         <v>15308</v>
@@ -1106,10 +1106,10 @@
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
         <v>18743</v>
@@ -1132,7 +1132,7 @@
         <v>29</v>
       </c>
       <c r="D31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" t="n">
         <v>29014</v>
@@ -1152,10 +1152,10 @@
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" t="n">
         <v>72223</v>
@@ -1175,10 +1175,10 @@
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D33" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" t="n">
         <v>81651</v>
@@ -1201,7 +1201,7 @@
         <v>100</v>
       </c>
       <c r="D34" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E34" t="n">
         <v>150368</v>
@@ -1221,10 +1221,10 @@
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D35" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E35" t="n">
         <v>85115</v>
@@ -1244,10 +1244,10 @@
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E36" t="n">
         <v>60939</v>
@@ -1270,7 +1270,7 @@
         <v>28</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" t="n">
         <v>21841</v>
@@ -1292,10 +1292,10 @@
         <v>5079</v>
       </c>
       <c r="C38" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
         <v>17390</v>
@@ -1320,7 +1320,7 @@
         <v>16</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E39" t="n">
         <v>15334</v>
@@ -1345,7 +1345,7 @@
         <v>14</v>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" t="n">
         <v>13968</v>
@@ -1370,7 +1370,7 @@
         <v>12</v>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" t="n">
         <v>10261</v>
@@ -1395,7 +1395,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E42" t="n">
         <v>14543</v>
@@ -1417,10 +1417,10 @@
         <v>7499</v>
       </c>
       <c r="C43" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
         <v>16505</v>
@@ -1442,10 +1442,10 @@
         <v>27675</v>
       </c>
       <c r="C44" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D44" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E44" t="n">
         <v>29905</v>
@@ -1467,10 +1467,10 @@
         <v>32388</v>
       </c>
       <c r="C45" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D45" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E45" t="n">
         <v>21251</v>
@@ -1492,10 +1492,10 @@
         <v>41375</v>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E46" t="n">
         <v>22844</v>
@@ -1517,10 +1517,10 @@
         <v>51183</v>
       </c>
       <c r="C47" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E47" t="n">
         <v>24239</v>
@@ -1542,10 +1542,10 @@
         <v>30354</v>
       </c>
       <c r="C48" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E48" t="n">
         <v>18976</v>
@@ -1570,7 +1570,7 @@
         <v>17</v>
       </c>
       <c r="D49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E49" t="n">
         <v>10532</v>
@@ -1595,7 +1595,7 @@
         <v>13</v>
       </c>
       <c r="D50" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E50" t="n">
         <v>9411</v>
@@ -1617,10 +1617,10 @@
         <v>3806</v>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E51" t="n">
         <v>5840</v>
@@ -1670,7 +1670,7 @@
         <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
         <v>4519</v>
@@ -1695,7 +1695,7 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E54" t="n">
         <v>7995</v>
@@ -1720,7 +1720,7 @@
         <v>13</v>
       </c>
       <c r="D55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E55" t="n">
         <v>7501</v>
@@ -1745,7 +1745,7 @@
         <v>18</v>
       </c>
       <c r="D56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E56" t="n">
         <v>7643</v>
@@ -1767,10 +1767,10 @@
         <v>14303</v>
       </c>
       <c r="C57" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
         <v>9983</v>
@@ -1792,10 +1792,10 @@
         <v>18803</v>
       </c>
       <c r="C58" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D58" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
         <v>7044</v>
@@ -1820,7 +1820,7 @@
         <v>21</v>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E59" t="n">
         <v>6021</v>
@@ -1845,7 +1845,7 @@
         <v>18</v>
       </c>
       <c r="D60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E60" t="n">
         <v>5358</v>
@@ -1870,7 +1870,7 @@
         <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E61" t="n">
         <v>3621</v>
@@ -1920,7 +1920,7 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E63" t="n">
         <v>1960</v>
@@ -1945,7 +1945,7 @@
         <v>7</v>
       </c>
       <c r="D64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E64" t="n">
         <v>2515</v>
@@ -1970,7 +1970,7 @@
         <v>6</v>
       </c>
       <c r="D65" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E65" t="n">
         <v>2432</v>
@@ -1995,7 +1995,7 @@
         <v>6</v>
       </c>
       <c r="D66" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E66" t="n">
         <v>3462</v>
@@ -2061,10 +2061,10 @@
         <v>13610</v>
       </c>
       <c r="C69" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D69" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E69" t="n">
         <v>4067</v>
@@ -2081,14 +2081,35 @@
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>28</v>
+      </c>
+      <c r="D70" t="n">
+        <v>14</v>
+      </c>
       <c r="E70" t="n">
-        <v>170</v>
+        <v>5375</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="n">
-        <v>74</v>
+        <v>1771</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>157</v>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="n">
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>